<commit_message>
Correção TAGS nas tasks
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gusta\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00AF4B42-371F-45FF-ABCA-68DB73400F1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C52C0CDF-4E9F-445B-B44F-2B784D7DA8BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23220" yWindow="10620" windowWidth="21500" windowHeight="13250" xr2:uid="{7D0B843E-6FC6-4887-A400-5996755EC944}"/>
+    <workbookView xWindow="-23540" yWindow="10720" windowWidth="21500" windowHeight="13250" xr2:uid="{7D0B843E-6FC6-4887-A400-5996755EC944}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3002" uniqueCount="1011">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3092" uniqueCount="1011">
   <si>
     <t>ID</t>
   </si>
@@ -3526,7 +3526,7 @@
   <dimension ref="A1:N335"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="32.85546875" customWidth="1"/>
+    <col min="3" max="3" width="39.42578125" customWidth="1"/>
     <col min="5" max="5" width="29.5703125" customWidth="1"/>
     <col min="6" max="6" width="26.140625" customWidth="1"/>
   </cols>
@@ -10986,7 +10986,9 @@
       <c r="F170" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G170" s="2"/>
+      <c r="G170" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H170" s="2">
         <v>11664</v>
       </c>
@@ -11028,7 +11030,9 @@
       <c r="F171" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="G171" s="5"/>
+      <c r="G171" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H171" s="5">
         <v>11626</v>
       </c>
@@ -11070,7 +11074,9 @@
       <c r="F172" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G172" s="2"/>
+      <c r="G172" s="2" t="s">
+        <v>45</v>
+      </c>
       <c r="H172" s="2">
         <v>11629</v>
       </c>
@@ -11112,7 +11118,9 @@
       <c r="F173" s="2" t="s">
         <v>562</v>
       </c>
-      <c r="G173" s="2"/>
+      <c r="G173" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="H173" s="2">
         <v>11635</v>
       </c>
@@ -11154,7 +11162,9 @@
       <c r="F174" s="2" t="s">
         <v>562</v>
       </c>
-      <c r="G174" s="2"/>
+      <c r="G174" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="H174" s="2">
         <v>11635</v>
       </c>
@@ -11196,7 +11206,9 @@
       <c r="F175" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="G175" s="5"/>
+      <c r="G175" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H175" s="5">
         <v>11811</v>
       </c>
@@ -11238,7 +11250,9 @@
       <c r="F176" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="G176" s="2"/>
+      <c r="G176" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H176" s="2">
         <v>11696</v>
       </c>
@@ -11280,7 +11294,9 @@
       <c r="F177" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="G177" s="5"/>
+      <c r="G177" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H177" s="5">
         <v>11696</v>
       </c>
@@ -11322,7 +11338,9 @@
       <c r="F178" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="G178" s="2"/>
+      <c r="G178" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H178" s="2">
         <v>11809</v>
       </c>
@@ -11364,7 +11382,9 @@
       <c r="F179" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="G179" s="5"/>
+      <c r="G179" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="H179" s="5">
         <v>11830</v>
       </c>
@@ -11406,7 +11426,9 @@
       <c r="F180" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="G180" s="2"/>
+      <c r="G180" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="H180" s="2">
         <v>11830</v>
       </c>
@@ -11448,7 +11470,9 @@
       <c r="F181" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="G181" s="5"/>
+      <c r="G181" s="5" t="s">
+        <v>24</v>
+      </c>
       <c r="H181" s="5">
         <v>11841</v>
       </c>
@@ -11490,7 +11514,9 @@
       <c r="F182" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="G182" s="2"/>
+      <c r="G182" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="H182" s="2">
         <v>11841</v>
       </c>
@@ -11532,7 +11558,9 @@
       <c r="F183" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="G183" s="5"/>
+      <c r="G183" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H183" s="5">
         <v>12001</v>
       </c>
@@ -11574,7 +11602,9 @@
       <c r="F184" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G184" s="2"/>
+      <c r="G184" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H184" s="2">
         <v>12032</v>
       </c>
@@ -11616,7 +11646,9 @@
       <c r="F185" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="G185" s="5"/>
+      <c r="G185" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H185" s="5">
         <v>12040</v>
       </c>
@@ -11658,7 +11690,9 @@
       <c r="F186" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G186" s="2"/>
+      <c r="G186" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H186" s="2">
         <v>12096</v>
       </c>
@@ -11700,7 +11734,9 @@
       <c r="F187" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="G187" s="5"/>
+      <c r="G187" s="5" t="s">
+        <v>65</v>
+      </c>
       <c r="H187" s="5">
         <v>12226</v>
       </c>
@@ -11742,7 +11778,9 @@
       <c r="F188" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G188" s="2"/>
+      <c r="G188" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H188" s="2">
         <v>11953</v>
       </c>
@@ -11784,7 +11822,9 @@
       <c r="F189" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="G189" s="5"/>
+      <c r="G189" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H189" s="5">
         <v>11953</v>
       </c>
@@ -11826,7 +11866,9 @@
       <c r="F190" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G190" s="2"/>
+      <c r="G190" s="2" t="s">
+        <v>45</v>
+      </c>
       <c r="H190" s="2">
         <v>11917</v>
       </c>
@@ -11868,7 +11910,9 @@
       <c r="F191" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="G191" s="5"/>
+      <c r="G191" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="H191" s="5">
         <v>11917</v>
       </c>
@@ -11910,7 +11954,9 @@
       <c r="F192" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="G192" s="2"/>
+      <c r="G192" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="H192" s="2">
         <v>12099</v>
       </c>
@@ -11952,7 +11998,9 @@
       <c r="F193" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="G193" s="5"/>
+      <c r="G193" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="H193" s="5">
         <v>12099</v>
       </c>
@@ -11994,7 +12042,9 @@
       <c r="F194" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="G194" s="2"/>
+      <c r="G194" s="2" t="s">
+        <v>45</v>
+      </c>
       <c r="H194" s="2">
         <v>12165</v>
       </c>
@@ -12036,7 +12086,9 @@
       <c r="F195" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="G195" s="5"/>
+      <c r="G195" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H195" s="5">
         <v>11898</v>
       </c>
@@ -12078,7 +12130,9 @@
       <c r="F196" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G196" s="2"/>
+      <c r="G196" s="2" t="s">
+        <v>45</v>
+      </c>
       <c r="H196" s="2">
         <v>12260</v>
       </c>
@@ -12120,7 +12174,9 @@
       <c r="F197" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="G197" s="5"/>
+      <c r="G197" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H197" s="5">
         <v>11778</v>
       </c>
@@ -12162,7 +12218,9 @@
       <c r="F198" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="G198" s="2"/>
+      <c r="G198" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="H198" s="2">
         <v>12101</v>
       </c>
@@ -12204,7 +12262,9 @@
       <c r="F199" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="G199" s="5"/>
+      <c r="G199" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="H199" s="5">
         <v>12101</v>
       </c>
@@ -12246,7 +12306,9 @@
       <c r="F200" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="G200" s="2"/>
+      <c r="G200" s="2" t="s">
+        <v>45</v>
+      </c>
       <c r="H200" s="2">
         <v>11838</v>
       </c>
@@ -12288,7 +12350,9 @@
       <c r="F201" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="G201" s="5"/>
+      <c r="G201" s="2" t="s">
+        <v>45</v>
+      </c>
       <c r="H201" s="5">
         <v>11838</v>
       </c>
@@ -12330,7 +12394,9 @@
       <c r="F202" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="G202" s="2"/>
+      <c r="G202" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H202" s="2">
         <v>11916</v>
       </c>
@@ -12372,7 +12438,9 @@
       <c r="F203" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="G203" s="5"/>
+      <c r="G203" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="H203" s="5">
         <v>12163</v>
       </c>
@@ -12414,7 +12482,9 @@
       <c r="F204" s="2" t="s">
         <v>562</v>
       </c>
-      <c r="G204" s="2"/>
+      <c r="G204" s="2" t="s">
+        <v>103</v>
+      </c>
       <c r="H204" s="2">
         <v>12174</v>
       </c>
@@ -12456,7 +12526,9 @@
       <c r="F205" s="5" t="s">
         <v>562</v>
       </c>
-      <c r="G205" s="5"/>
+      <c r="G205" s="5" t="s">
+        <v>103</v>
+      </c>
       <c r="H205" s="5">
         <v>12174</v>
       </c>
@@ -12498,7 +12570,9 @@
       <c r="F206" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G206" s="2"/>
+      <c r="G206" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H206" s="2">
         <v>12111</v>
       </c>
@@ -12540,7 +12614,9 @@
       <c r="F207" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="G207" s="5"/>
+      <c r="G207" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H207" s="5">
         <v>12111</v>
       </c>
@@ -12582,7 +12658,9 @@
       <c r="F208" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="G208" s="2"/>
+      <c r="G208" s="2" t="s">
+        <v>103</v>
+      </c>
       <c r="H208" s="2">
         <v>12360</v>
       </c>
@@ -12624,7 +12702,9 @@
       <c r="F209" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="G209" s="5"/>
+      <c r="G209" s="2" t="s">
+        <v>103</v>
+      </c>
       <c r="H209" s="5">
         <v>12360</v>
       </c>
@@ -12666,7 +12746,9 @@
       <c r="F210" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G210" s="2"/>
+      <c r="G210" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H210" s="2">
         <v>12401</v>
       </c>
@@ -12708,7 +12790,9 @@
       <c r="F211" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="G211" s="5"/>
+      <c r="G211" s="5" t="s">
+        <v>103</v>
+      </c>
       <c r="H211" s="5">
         <v>12320</v>
       </c>
@@ -12750,7 +12834,9 @@
       <c r="F212" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="G212" s="2"/>
+      <c r="G212" s="5" t="s">
+        <v>103</v>
+      </c>
       <c r="H212" s="2">
         <v>12320</v>
       </c>
@@ -12792,7 +12878,9 @@
       <c r="F213" s="5" t="s">
         <v>667</v>
       </c>
-      <c r="G213" s="5"/>
+      <c r="G213" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="H213" s="5">
         <v>12243</v>
       </c>
@@ -12834,7 +12922,9 @@
       <c r="F214" s="2" t="s">
         <v>667</v>
       </c>
-      <c r="G214" s="2"/>
+      <c r="G214" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="H214" s="2">
         <v>12243</v>
       </c>
@@ -12964,7 +13054,9 @@
       <c r="F217" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="G217" s="5"/>
+      <c r="G217" s="5" t="s">
+        <v>24</v>
+      </c>
       <c r="H217" s="5">
         <v>11844</v>
       </c>
@@ -13006,7 +13098,9 @@
       <c r="F218" s="2" t="s">
         <v>667</v>
       </c>
-      <c r="G218" s="2"/>
+      <c r="G218" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H218" s="2">
         <v>12403</v>
       </c>
@@ -13048,7 +13142,9 @@
       <c r="F219" s="5" t="s">
         <v>667</v>
       </c>
-      <c r="G219" s="5"/>
+      <c r="G219" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H219" s="5">
         <v>12403</v>
       </c>
@@ -13090,7 +13186,9 @@
       <c r="F220" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="G220" s="2"/>
+      <c r="G220" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H220" s="2">
         <v>12452</v>
       </c>
@@ -13132,7 +13230,9 @@
       <c r="F221" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="G221" s="5"/>
+      <c r="G221" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H221" s="5">
         <v>12452</v>
       </c>
@@ -13174,7 +13274,9 @@
       <c r="F222" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="G222" s="2"/>
+      <c r="G222" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H222" s="2">
         <v>12479</v>
       </c>
@@ -13216,7 +13318,9 @@
       <c r="F223" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="G223" s="5"/>
+      <c r="G223" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="H223" s="5">
         <v>12982</v>
       </c>
@@ -13258,7 +13362,9 @@
       <c r="F224" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="G224" s="2"/>
+      <c r="G224" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H224" s="2">
         <v>12888</v>
       </c>
@@ -13300,7 +13406,9 @@
       <c r="F225" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="G225" s="5"/>
+      <c r="G225" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H225" s="5">
         <v>12966</v>
       </c>
@@ -13342,7 +13450,9 @@
       <c r="F226" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="G226" s="2"/>
+      <c r="G226" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H226" s="2">
         <v>12886</v>
       </c>
@@ -13384,7 +13494,9 @@
       <c r="F227" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="G227" s="5"/>
+      <c r="G227" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H227" s="5">
         <v>12890</v>
       </c>
@@ -13426,7 +13538,9 @@
       <c r="F228" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="G228" s="2"/>
+      <c r="G228" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H228" s="2">
         <v>12940</v>
       </c>
@@ -13468,7 +13582,9 @@
       <c r="F229" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="G229" s="5"/>
+      <c r="G229" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H229" s="5">
         <v>12988</v>
       </c>
@@ -13510,7 +13626,9 @@
       <c r="F230" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="G230" s="2"/>
+      <c r="G230" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H230" s="2">
         <v>12988</v>
       </c>
@@ -13552,7 +13670,9 @@
       <c r="F231" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="G231" s="5"/>
+      <c r="G231" s="5" t="s">
+        <v>103</v>
+      </c>
       <c r="H231" s="5">
         <v>13081</v>
       </c>
@@ -13594,7 +13714,9 @@
       <c r="F232" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="G232" s="2"/>
+      <c r="G232" s="5" t="s">
+        <v>103</v>
+      </c>
       <c r="H232" s="2">
         <v>13081</v>
       </c>
@@ -13680,7 +13802,9 @@
       <c r="F234" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="G234" s="2"/>
+      <c r="G234" s="2" t="s">
+        <v>103</v>
+      </c>
       <c r="H234" s="2">
         <v>13128</v>
       </c>
@@ -13722,7 +13846,9 @@
       <c r="F235" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="G235" s="5"/>
+      <c r="G235" s="2" t="s">
+        <v>103</v>
+      </c>
       <c r="H235" s="5">
         <v>13119</v>
       </c>
@@ -13764,7 +13890,9 @@
       <c r="F236" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="G236" s="2"/>
+      <c r="G236" s="2" t="s">
+        <v>103</v>
+      </c>
       <c r="H236" s="2">
         <v>13119</v>
       </c>
@@ -13806,7 +13934,9 @@
       <c r="F237" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="G237" s="5"/>
+      <c r="G237" s="2" t="s">
+        <v>103</v>
+      </c>
       <c r="H237" s="5">
         <v>13136</v>
       </c>
@@ -13848,7 +13978,9 @@
       <c r="F238" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="G238" s="2"/>
+      <c r="G238" s="2" t="s">
+        <v>103</v>
+      </c>
       <c r="H238" s="2">
         <v>13136</v>
       </c>
@@ -13890,7 +14022,9 @@
       <c r="F239" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="G239" s="5"/>
+      <c r="G239" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="H239" s="5">
         <v>11852</v>
       </c>
@@ -13976,7 +14110,9 @@
       <c r="F241" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="G241" s="5"/>
+      <c r="G241" s="2" t="s">
+        <v>103</v>
+      </c>
       <c r="H241" s="5">
         <v>11852</v>
       </c>
@@ -14150,7 +14286,9 @@
       <c r="F245" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="G245" s="5"/>
+      <c r="G245" s="2" t="s">
+        <v>103</v>
+      </c>
       <c r="H245" s="5">
         <v>12640</v>
       </c>
@@ -14192,7 +14330,9 @@
       <c r="F246" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G246" s="2"/>
+      <c r="G246" s="2" t="s">
+        <v>45</v>
+      </c>
       <c r="H246" s="2">
         <v>13380</v>
       </c>
@@ -14234,7 +14374,9 @@
       <c r="F247" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="G247" s="5"/>
+      <c r="G247" s="2" t="s">
+        <v>45</v>
+      </c>
       <c r="H247" s="5">
         <v>13380</v>
       </c>
@@ -14276,7 +14418,9 @@
       <c r="F248" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G248" s="2"/>
+      <c r="G248" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="H248" s="2">
         <v>10206</v>
       </c>
@@ -14318,7 +14462,9 @@
       <c r="F249" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="G249" s="2"/>
+      <c r="G249" s="2" t="s">
+        <v>250</v>
+      </c>
       <c r="H249" s="2">
         <v>13566</v>
       </c>
@@ -14448,7 +14594,9 @@
       <c r="F252" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="G252" s="5"/>
+      <c r="G252" s="2" t="s">
+        <v>250</v>
+      </c>
       <c r="H252" s="5">
         <v>13335</v>
       </c>
@@ -14490,7 +14638,9 @@
       <c r="F253" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="G253" s="2"/>
+      <c r="G253" s="2" t="s">
+        <v>250</v>
+      </c>
       <c r="H253" s="2">
         <v>13335</v>
       </c>
@@ -14532,7 +14682,9 @@
       <c r="F254" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="G254" s="5"/>
+      <c r="G254" s="5" t="s">
+        <v>103</v>
+      </c>
       <c r="H254" s="5">
         <v>13130</v>
       </c>
@@ -14574,7 +14726,9 @@
       <c r="F255" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="G255" s="2"/>
+      <c r="G255" s="5" t="s">
+        <v>103</v>
+      </c>
       <c r="H255" s="2">
         <v>13130</v>
       </c>
@@ -14616,7 +14770,9 @@
       <c r="F256" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="G256" s="5"/>
+      <c r="G256" s="5" t="s">
+        <v>103</v>
+      </c>
       <c r="H256" s="5">
         <v>13122</v>
       </c>
@@ -14658,7 +14814,9 @@
       <c r="F257" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="G257" s="2"/>
+      <c r="G257" s="5" t="s">
+        <v>103</v>
+      </c>
       <c r="H257" s="2">
         <v>13122</v>
       </c>
@@ -14700,7 +14858,9 @@
       <c r="F258" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="G258" s="5"/>
+      <c r="G258" s="5" t="s">
+        <v>103</v>
+      </c>
       <c r="H258" s="5">
         <v>13125</v>
       </c>
@@ -14742,7 +14902,9 @@
       <c r="F259" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="G259" s="2"/>
+      <c r="G259" s="5" t="s">
+        <v>103</v>
+      </c>
       <c r="H259" s="2">
         <v>13125</v>
       </c>
@@ -14784,7 +14946,9 @@
       <c r="F260" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="G260" s="5"/>
+      <c r="G260" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="H260" s="5">
         <v>13502</v>
       </c>
@@ -14826,7 +14990,9 @@
       <c r="F261" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G261" s="2"/>
+      <c r="G261" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="H261" s="2">
         <v>13502</v>
       </c>
@@ -14868,7 +15034,9 @@
       <c r="F262" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="G262" s="5"/>
+      <c r="G262" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H262" s="5">
         <v>13354</v>
       </c>
@@ -14910,7 +15078,9 @@
       <c r="F263" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G263" s="2"/>
+      <c r="G263" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H263" s="2">
         <v>13354</v>
       </c>
@@ -14952,7 +15122,9 @@
       <c r="F264" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="G264" s="5"/>
+      <c r="G264" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="H264" s="5">
         <v>13098</v>
       </c>
@@ -14994,7 +15166,9 @@
       <c r="F265" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="G265" s="2"/>
+      <c r="G265" s="2" t="s">
+        <v>45</v>
+      </c>
       <c r="H265" s="2">
         <v>13098</v>
       </c>
@@ -15212,7 +15386,9 @@
       <c r="F270" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="G270" s="5"/>
+      <c r="G270" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="H270" s="5">
         <v>13571</v>
       </c>
@@ -15254,7 +15430,9 @@
       <c r="F271" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G271" s="2"/>
+      <c r="G271" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="H271" s="2">
         <v>13571</v>
       </c>
@@ -16968,7 +17146,9 @@
       <c r="F310" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G310" s="2"/>
+      <c r="G310" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="H310" s="2">
         <v>14402</v>
       </c>

</xml_diff>